<commit_message>
Web tools data: make barcode 3 the positive sample instead of 11
Relabel 123456789-11 -> 123456789-3 across the linked files so the second
culture-positive water sample is barcode 3 (barcode 9 unchanged):
- lab_results.xlsx: sample 3 -> K. pneumoniae, sample 11 -> negative
- genomes/123456789-11.fasta renamed to 123456789-3.fasta (same genome)
- mlst-Pasteur.csv and tree.nwk relabelled to 123456789-3

All four files cross-check to the same positives (3, 9).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/course_data_2026/Web_tools/data/lab_results.xlsx
+++ b/course_data_2026/Web_tools/data/lab_results.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>negative</t>
+          <t>K. pneumoniae</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>K. pneumoniae</t>
+          <t>negative</t>
         </is>
       </c>
     </row>

</xml_diff>